<commit_message>
Search by barcode: the register and merchant app find items by any barcode they ring under (whole, with or without a leading 0, or the last digits), whole-barcode matches first, and show the code on every result; price check and the item editor list every barcode; search cached per catalog (5-17 ms on 9,284 items); merchant list capped at 200 rows; tester cases R52 and M38
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adpay-pos-test-plan.xlsx
+++ b/docs/adpay-pos-test-plan.xlsx
@@ -1060,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2557,6 +2557,34 @@
       <c r="E62" s="13" t="n"/>
       <c r="F62" s="13" t="n"/>
     </row>
+    <row r="63" ht="143" customHeight="1">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>R52</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Find an item by typing its barcode</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>1. Click the search box and type 200000100131 (don't press Enter). Look at the tile.
+2. Replace it with just 0131. Look at the tile.
+3. Replace it with coffee.
+4. Clear the search. Press Price check, tap Hot Coffee — Medium, read the box, press Done, then Price check again to turn it off.</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
+        <is>
+          <t>⚑ Worked out from the code, not yet clicked through by us. If it's different, report it anyway: the mistake may be ours.
+The whole barcode finds exactly one tile, Hot Coffee — Medium, with "✓ 200000100131" in bold under the name. With 0131 the same tile shows the barcode with its last four digits in bold. With coffee, each coffee tile shows its own barcode (e.g. 200000100148 for Large). Price check shows the barcode under the item name. (Pressing Enter after a whole barcode rings it, exactly like a scan.)</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="n"/>
+      <c r="F63" s="13" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
@@ -2568,7 +2596,7 @@
     <mergeCell ref="A7:F7"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E5 E6 E8 E9 E10 E11 E12 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E38 E39 E40 E41 E42 E43 E44 E46 E47 E48 E49 E50 E51 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Pass, Fail or Skipped" prompt="Pass, Fail or Skipped" type="list">
+    <dataValidation sqref="E5 E6 E8 E9 E10 E11 E12 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E38 E39 E40 E41 E42 E43 E44 E46 E47 E48 E49 E50 E51 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Pass, Fail or Skipped" prompt="Pass, Fail or Skipped" type="list">
       <formula1>"Pass,Fail,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2583,7 +2611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3719,30 +3747,56 @@
       <c r="E51" s="13" t="n"/>
       <c r="F51" s="13" t="n"/>
     </row>
-    <row r="52" ht="75.5" customHeight="1">
+    <row r="52" ht="89" customHeight="1">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>M37</t>
+          <t>M38</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Uploading again never makes duplicates</t>
+          <t>Look an item up by barcode</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>1. Choose the same file again and press Preview. Don't import.</t>
+          <t>1. Items → Items. In the search box type 200000100131.
+2. Tap the row and look under "Barcode (UPC)".</t>
         </is>
       </c>
       <c r="D52" s="17" t="inlineStr">
         <is>
           <t>⚑ Worked out from the code, not yet clicked through by us. If it's different, report it anyway: the mistake may be ours.
-"Will import 12 of 12 items: 0 new, 0 updated, 12 unchanged." and Categories "… 0 new, 5 already in your catalog …".</t>
+One row, Hot Coffee — Medium, with "✓ Barcode 200000100131" under it (every row shows its barcode). The item shows 200000100131 in the Barcode (UPC) box.</t>
         </is>
       </c>
       <c r="E52" s="13" t="n"/>
       <c r="F52" s="13" t="n"/>
+    </row>
+    <row r="53" ht="75.5" customHeight="1">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>M37</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Uploading again never makes duplicates</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>1. Choose the same file again and press Preview. Don't import.</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>⚑ Worked out from the code, not yet clicked through by us. If it's different, report it anyway: the mistake may be ours.
+"Will import 12 of 12 items: 0 new, 0 updated, 12 unchanged." and Categories "… 0 new, 5 already in your catalog …".</t>
+        </is>
+      </c>
+      <c r="E53" s="13" t="n"/>
+      <c r="F53" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -3759,7 +3813,7 @@
     <mergeCell ref="A7:F7"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E5 E6 E8 E9 E10 E11 E12 E13 E14 E15 E16 E18 E19 E21 E22 E23 E24 E25 E26 E28 E29 E31 E32 E34 E35 E36 E37 E38 E39 E40 E41 E43 E44 E46 E47 E49 E50 E51 E52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Pass, Fail or Skipped" prompt="Pass, Fail or Skipped" type="list">
+    <dataValidation sqref="E5 E6 E8 E9 E10 E11 E12 E13 E14 E15 E16 E18 E19 E21 E22 E23 E24 E25 E26 E28 E29 E31 E32 E34 E35 E36 E37 E38 E39 E40 E41 E43 E44 E46 E47 E49 E50 E51 E52 E53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Pass, Fail or Skipped" prompt="Pass, Fail or Skipped" type="list">
       <formula1>"Pass,Fail,Skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>